<commit_message>
v2.0 - Major updates: Travel summary sheet, Hebrew sheet names, bidirectional distance lookup, consecutive duplicates removal
</commit_message>
<xml_diff>
--- a/Config.xlsx
+++ b/Config.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shmuel\.gemini\antigravity\scratch\Timesheet_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61A1C564-54B8-4355-A05B-7C8984064B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF19A816-C522-4751-99D2-16AF6CAC0D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="1" r:id="rId1"/>
     <sheet name="Settings" sheetId="2" r:id="rId2"/>
-    <sheet name="Distances" sheetId="3" r:id="rId3"/>
+    <sheet name="Adresses" sheetId="4" r:id="rId3"/>
+    <sheet name="Distances" sheetId="3" r:id="rId4"/>
+    <sheet name="גיליון1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,18 +37,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="68">
   <si>
     <t>Active</t>
   </si>
   <si>
+    <t>Adress</t>
+  </si>
+  <si>
+    <t>אור</t>
+  </si>
+  <si>
+    <t>אשד 1 צור הדסה</t>
+  </si>
+  <si>
+    <t>דרור</t>
+  </si>
+  <si>
+    <t>רימון 2 בר גיורא</t>
+  </si>
+  <si>
+    <t>מעיינות</t>
+  </si>
+  <si>
+    <t>דפנה 2 צור הדסה</t>
+  </si>
+  <si>
+    <t>נווה יעקב</t>
+  </si>
+  <si>
+    <t>מינהל קהילתי נווה יעקב</t>
+  </si>
+  <si>
+    <t>שערי רחמים</t>
+  </si>
+  <si>
+    <t>מיכל 7, ירושלים</t>
+  </si>
+  <si>
+    <t>שראל</t>
+  </si>
+  <si>
+    <t>צור 5 מבשרת</t>
+  </si>
+  <si>
     <t>Value</t>
   </si>
   <si>
     <t>Key</t>
   </si>
   <si>
-    <t>בית (כפר אלדד)</t>
+    <t>בית</t>
   </si>
   <si>
     <t>Home_Location</t>
@@ -61,31 +102,145 @@
     <t>מרחק (ק"מ)</t>
   </si>
   <si>
-    <t>אור</t>
-  </si>
-  <si>
-    <t>דרור</t>
-  </si>
-  <si>
-    <t>מעיינות</t>
-  </si>
-  <si>
     <t>חנות</t>
   </si>
   <si>
-    <t>נווה יעקב</t>
-  </si>
-  <si>
-    <t>בית</t>
-  </si>
-  <si>
-    <t>כללי</t>
-  </si>
-  <si>
-    <t>שערי רחמים</t>
-  </si>
-  <si>
-    <t>שראל</t>
+    <t>הקרן לידידות</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>יד חרוצים 10, ירושלים</t>
+  </si>
+  <si>
+    <t>דם המכבים 28 מודיעין</t>
+  </si>
+  <si>
+    <t>בית טכמן</t>
+  </si>
+  <si>
+    <t>חוגלה 8 צור הדסה</t>
+  </si>
+  <si>
+    <t>הערות למסלול</t>
+  </si>
+  <si>
+    <t>נסיעה פנימית בתוך צור הדסה</t>
+  </si>
+  <si>
+    <t>נסיעה לבר גיורא (כביש 375)</t>
+  </si>
+  <si>
+    <t>דרך כביש המנהרות לאזור תעשיה תלפיות</t>
+  </si>
+  <si>
+    <t>דרך כביש בגין לרוממה</t>
+  </si>
+  <si>
+    <t>דרך עין כרם או בגין/כביש 1 למבשרת</t>
+  </si>
+  <si>
+    <t>חציית ירושלים (בגין צפון)</t>
+  </si>
+  <si>
+    <t>דרך בית שמש (38) או כביש 1 למודיעין</t>
+  </si>
+  <si>
+    <t>בתוך צור הדסה</t>
+  </si>
+  <si>
+    <t>יציאה מצור הדסה לבר גיורא</t>
+  </si>
+  <si>
+    <t>תלפיות</t>
+  </si>
+  <si>
+    <t>מבשרת ציון</t>
+  </si>
+  <si>
+    <t>רוממה</t>
+  </si>
+  <si>
+    <t>מודיעין</t>
+  </si>
+  <si>
+    <t>מבר גיורא לצור הדסה</t>
+  </si>
+  <si>
+    <t>דרך המנהרות לתלפיות</t>
+  </si>
+  <si>
+    <t>למבשרת</t>
+  </si>
+  <si>
+    <t>לרוממה</t>
+  </si>
+  <si>
+    <t>לנווה יעקב</t>
+  </si>
+  <si>
+    <t>למודיעין</t>
+  </si>
+  <si>
+    <t>לתלפיות</t>
+  </si>
+  <si>
+    <t>מתלפיות למבשרת (דרך בגין)</t>
+  </si>
+  <si>
+    <t>בתוך ירושלים</t>
+  </si>
+  <si>
+    <t>מתלפיות לנווה יעקב</t>
+  </si>
+  <si>
+    <t>מתלפיות למודיעין (דרך 443)</t>
+  </si>
+  <si>
+    <t>ממבשרת לכניסה לעיר/רוממה</t>
+  </si>
+  <si>
+    <t>ממבשרת לנווה יעקב (דרך יגאל ידין)</t>
+  </si>
+  <si>
+    <t>ממבשרת למודיעין (כביש 1 + 443)</t>
+  </si>
+  <si>
+    <t>מרוממה לנווה יעקב</t>
+  </si>
+  <si>
+    <t>מירושלים למודיעין</t>
+  </si>
+  <si>
+    <t>מנווה יעקב למודיעין (443)</t>
+  </si>
+  <si>
+    <t>דרך הר חומה לתלפיות (יד חרוצים)</t>
+  </si>
+  <si>
+    <t>דרך דרך חברון/בגין לרוממה</t>
+  </si>
+  <si>
+    <t>דרך בגין וכביש 1 למבשרת</t>
+  </si>
+  <si>
+    <t>חציית ירושלים (דרך בגין צפון או דרך העופל/כביש 1)</t>
+  </si>
+  <si>
+    <t>דרך כביש המנהרות (60) וצומת חוסאן (375) לצור הדסה</t>
+  </si>
+  <si>
+    <t>אותה דרך לצור הדסה</t>
+  </si>
+  <si>
+    <t>דרך כביש המנהרות ופניה לנס הרים/בר גיורא</t>
+  </si>
+  <si>
+    <t>דרך ירושלים (בגין) וכביש 443 למודיעין</t>
+  </si>
+  <si>
+    <t>עלי דפנה 104 נוקדים</t>
   </si>
 </sst>
 </file>
@@ -178,10 +333,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
+      <alignment vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1" indent="1" readingOrder="2"/>
+      <alignment vertical="center" wrapText="1" readingOrder="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -487,50 +642,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="B5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>16</v>
+      <c r="B7" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -540,23 +712,128 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D8E02F0-B710-4BAE-94DD-11A691A04581}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -564,195 +841,670 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="21.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1.3</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2">
+        <v>18.5</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2">
+        <v>23</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2">
+        <v>25.5</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="3">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
+      <c r="C8" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2">
+        <v>43</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1.5</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="2">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="2">
+        <v>17.8</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2">
+        <v>24.5</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="2">
+        <v>22.5</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3">
-        <v>26.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
+      <c r="C15" s="2">
+        <v>32.5</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="2">
+        <v>42.5</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="2">
+        <v>19.5</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="2">
+        <v>26</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3">
-        <v>2.2000000000000002</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="2" t="s">
+      <c r="C20" s="2">
+        <v>24</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C21" s="2">
+        <v>34</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="2">
+        <v>44</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2">
+        <v>18</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="3">
-        <v>38.9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
+      <c r="C24" s="2">
+        <v>25</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="2">
+        <v>22.8</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="3">
-        <v>29.7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="3">
-        <v>23.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="2" t="s">
+      <c r="C26" s="2">
+        <v>33</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C27" s="2">
+        <v>43</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" s="2">
+        <v>13.5</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="3">
-        <v>3.4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="C29" s="2">
+        <v>8.5</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="2">
+        <v>16.5</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="2">
+        <v>36</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="3">
-        <v>35.4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="3">
-        <v>30.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="3">
+      <c r="C32" s="2">
+        <v>6.5</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="2">
+        <v>15</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C34" s="2">
+        <v>27</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" s="2">
+        <v>10.5</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="2">
+        <v>31</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C37" s="2">
+        <v>33</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" s="2">
+        <v>14.5</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="2">
+        <v>23.5</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A40" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="2">
+        <v>29.5</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="2">
+        <v>32</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="3">
-        <v>13.4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="3">
-        <v>15.9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="3">
-        <v>38.1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="3">
-        <v>28.9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="3">
-        <v>27.2</v>
+      <c r="C42" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C43" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A44" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C44" s="2">
+        <v>33.5</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A45" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="2">
+        <v>30.5</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A46" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C46" s="2">
+        <v>54</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C40">
-    <sortCondition ref="A1:A40"/>
-  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{755F3197-7CDF-41CA-A6D4-63F5004265E4}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>